<commit_message>
1. Fix url and xml for Jie Xiong. 2. Delete duplicate data for Chen Change Loy
</commit_message>
<xml_diff>
--- a/Faculty.xlsx
+++ b/Faculty.xlsx
@@ -280,7 +280,7 @@
     <t>Jie Xiong</t>
   </si>
   <si>
-    <t>https://dblp.org/pid/62/2078.html</t>
+    <t>https://dblp.org/pid/75/198-1.html</t>
   </si>
   <si>
     <t>Joty Shafiq Rayhan</t>
@@ -1923,8 +1923,8 @@
       <c r="E32" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F32" s="6" t="s">
-        <v>31</v>
+      <c r="F32" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="G32" s="3"/>
       <c r="H32" s="12"/>

</xml_diff>